<commit_message>
docs: atualiza o arquivo burndown.xlsx com novas informações
</commit_message>
<xml_diff>
--- a/DOCS/burndown.xlsx
+++ b/DOCS/burndown.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\FATEC\sem3\API-3\DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE488731-C3FC-4EC7-A54C-4FFD63C0F4DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{346C36AF-E7E1-47E3-AEE2-5D1BC7244F32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Burn1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>Total de horas</t>
   </si>
@@ -148,6 +148,9 @@
   </si>
   <si>
     <t>T-14</t>
+  </si>
+  <si>
+    <t>Horas pendentes</t>
   </si>
 </sst>
 </file>
@@ -270,7 +273,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -278,26 +281,51 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="25">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -905,72 +933,72 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Burn1!$B$25:$V$25</c:f>
+              <c:f>Burn1!$B$16:$V$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>83</c:v>
+                  <c:v>74</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>73</c:v>
+                  <c:v>64</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>70</c:v>
+                  <c:v>61</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>67</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>60</c:v>
+                  <c:v>51</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>59</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>59</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>58</c:v>
+                  <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>48</c:v>
+                  <c:v>37.5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>48</c:v>
+                  <c:v>30.5</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>48</c:v>
+                  <c:v>29.5</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>48</c:v>
+                  <c:v>24.5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>48</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>48</c:v>
+                  <c:v>16.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>48</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>48</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>48</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>48</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>48</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>48</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>48</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1079,69 +1107,69 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Burn1!$B$26:$V$26</c:f>
+              <c:f>Burn1!$B$17:$V$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>83</c:v>
+                  <c:v>74</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>78.849999999999994</c:v>
+                  <c:v>70.3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>74.7</c:v>
+                  <c:v>66.599999999999994</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>70.55</c:v>
+                  <c:v>62.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>66.400000000000006</c:v>
+                  <c:v>59.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>62.25</c:v>
+                  <c:v>55.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>58.099999999999994</c:v>
+                  <c:v>51.8</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>53.949999999999996</c:v>
+                  <c:v>48.099999999999994</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>49.8</c:v>
+                  <c:v>44.4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>45.65</c:v>
+                  <c:v>40.699999999999996</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>41.5</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>37.349999999999994</c:v>
+                  <c:v>33.299999999999997</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>33.199999999999996</c:v>
+                  <c:v>29.599999999999994</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>29.049999999999997</c:v>
+                  <c:v>25.9</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>24.899999999999991</c:v>
+                  <c:v>22.199999999999996</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>20.749999999999993</c:v>
+                  <c:v>18.5</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>16.599999999999994</c:v>
+                  <c:v>14.799999999999997</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>12.449999999999989</c:v>
+                  <c:v>11.099999999999994</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>8.2999999999999972</c:v>
+                  <c:v>7.3999999999999915</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>4.1499999999999915</c:v>
+                  <c:v>3.7000000000000028</c:v>
                 </c:pt>
                 <c:pt idx="20">
                   <c:v>0</c:v>
@@ -1548,72 +1576,72 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Burn1!$B$25:$V$25</c:f>
+              <c:f>Burn1!$B$16:$V$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>83</c:v>
+                  <c:v>74</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>73</c:v>
+                  <c:v>64</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>70</c:v>
+                  <c:v>61</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>67</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>60</c:v>
+                  <c:v>51</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>59</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>59</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>58</c:v>
+                  <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>48</c:v>
+                  <c:v>37.5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>48</c:v>
+                  <c:v>30.5</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>48</c:v>
+                  <c:v>29.5</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>48</c:v>
+                  <c:v>24.5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>48</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>48</c:v>
+                  <c:v>16.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>48</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>48</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>48</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>48</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>48</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>48</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>48</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1722,69 +1750,69 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Burn1!$B$26:$V$26</c:f>
+              <c:f>Burn1!$B$17:$V$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>83</c:v>
+                  <c:v>74</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>78.849999999999994</c:v>
+                  <c:v>70.3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>74.7</c:v>
+                  <c:v>66.599999999999994</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>70.55</c:v>
+                  <c:v>62.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>66.400000000000006</c:v>
+                  <c:v>59.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>62.25</c:v>
+                  <c:v>55.5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>58.099999999999994</c:v>
+                  <c:v>51.8</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>53.949999999999996</c:v>
+                  <c:v>48.099999999999994</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>49.8</c:v>
+                  <c:v>44.4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>45.65</c:v>
+                  <c:v>40.699999999999996</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>41.5</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>37.349999999999994</c:v>
+                  <c:v>33.299999999999997</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>33.199999999999996</c:v>
+                  <c:v>29.599999999999994</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>29.049999999999997</c:v>
+                  <c:v>25.9</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>24.899999999999991</c:v>
+                  <c:v>22.199999999999996</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>20.749999999999993</c:v>
+                  <c:v>18.5</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>16.599999999999994</c:v>
+                  <c:v>14.799999999999997</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>12.449999999999989</c:v>
+                  <c:v>11.099999999999994</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>8.2999999999999972</c:v>
+                  <c:v>7.3999999999999915</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>4.1499999999999915</c:v>
+                  <c:v>3.7000000000000028</c:v>
                 </c:pt>
                 <c:pt idx="20">
                   <c:v>0</c:v>
@@ -2033,10 +2061,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>390524</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>14287</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>357867</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>144915</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6191250" cy="3638551"/>
     <xdr:graphicFrame macro="">
@@ -2104,31 +2132,34 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1884C1C-B0F0-42C1-9734-A26A7C746AC5}" name="Tabela2" displayName="Tabela2" ref="A1:V24" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="A1:V24" xr:uid="{E1884C1C-B0F0-42C1-9734-A26A7C746AC5}"/>
-  <tableColumns count="22">
-    <tableColumn id="1" xr3:uid="{DC2BAE98-3A26-4BC7-8ED6-C3303DF0038D}" name="Tasks" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{1A2025CD-23B1-415B-92B3-5881DCA18C20}" name="Total de horas" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{4BC0BD76-7741-45BB-97A7-D6882CC1F1D8}" name="Dia 1" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{00882AA1-DD73-47DC-8C10-EF217AC99768}" name="Dia 2" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{26CA22D1-FC01-468E-9640-E8C45E991335}" name="Dia 3" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{8637A8CA-1019-4007-B1C8-E2B239B9DDE1}" name="Dia 4" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{A817E580-DFE5-4C0E-95B3-BA357CCF9AE1}" name="Dia 5" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{D4E45274-3E12-45D7-8440-09BF785A95E4}" name="Dia 6" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{731C7356-2D40-41A5-B847-23C816E5BAD2}" name="Dia 7" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{824F84C5-6311-4AAA-96D8-D8FD71FBBAF6}" name="Dia 8" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{A41E8023-6BEE-4187-9A47-DA4E41991646}" name="Dia 9" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{FCCE3901-00D6-4E75-A167-FD4C20E71CF2}" name="Dia 10" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{E9D6ACAB-EF0B-42EB-977B-E157431B7C93}" name="Dia 11" dataDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{7DE82C8F-4251-435F-8119-4098379E7C92}" name="Dia 12" dataDxfId="8"/>
-    <tableColumn id="15" xr3:uid="{C0057573-93FA-4291-8B0E-84DA468004AA}" name="Dia 13" dataDxfId="7"/>
-    <tableColumn id="16" xr3:uid="{616A7614-87CD-480E-8FB6-B3E991E2E773}" name="Dia 14" dataDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{1EA39BE6-7D7D-43AD-8119-68FE10A2BB9C}" name="Dia 15" dataDxfId="5"/>
-    <tableColumn id="18" xr3:uid="{EF7A01F8-F878-4FFE-B140-126C702615BE}" name="Dia 16" dataDxfId="4"/>
-    <tableColumn id="19" xr3:uid="{9701BAD2-120F-49E8-9004-331E6F9C2716}" name="Dia 17" dataDxfId="3"/>
-    <tableColumn id="20" xr3:uid="{72A17F3E-6229-46C9-8FEE-BDF8B519F9FD}" name="Dia 18" dataDxfId="2"/>
-    <tableColumn id="21" xr3:uid="{1C3259A9-A4D5-488F-BE54-1D541CFA2C96}" name="Dia 19" dataDxfId="1"/>
-    <tableColumn id="22" xr3:uid="{4411E0A4-16AB-46BD-886B-34DA12503542}" name="Dia 20" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1884C1C-B0F0-42C1-9734-A26A7C746AC5}" name="Tabela2" displayName="Tabela2" ref="A1:W15" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+  <autoFilter ref="A1:W15" xr:uid="{E1884C1C-B0F0-42C1-9734-A26A7C746AC5}"/>
+  <tableColumns count="23">
+    <tableColumn id="1" xr3:uid="{DC2BAE98-3A26-4BC7-8ED6-C3303DF0038D}" name="Tasks" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{1A2025CD-23B1-415B-92B3-5881DCA18C20}" name="Total de horas" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{4BC0BD76-7741-45BB-97A7-D6882CC1F1D8}" name="Dia 1" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{00882AA1-DD73-47DC-8C10-EF217AC99768}" name="Dia 2" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{26CA22D1-FC01-468E-9640-E8C45E991335}" name="Dia 3" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{8637A8CA-1019-4007-B1C8-E2B239B9DDE1}" name="Dia 4" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{A817E580-DFE5-4C0E-95B3-BA357CCF9AE1}" name="Dia 5" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{D4E45274-3E12-45D7-8440-09BF785A95E4}" name="Dia 6" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{731C7356-2D40-41A5-B847-23C816E5BAD2}" name="Dia 7" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{824F84C5-6311-4AAA-96D8-D8FD71FBBAF6}" name="Dia 8" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{A41E8023-6BEE-4187-9A47-DA4E41991646}" name="Dia 9" dataDxfId="12"/>
+    <tableColumn id="12" xr3:uid="{FCCE3901-00D6-4E75-A167-FD4C20E71CF2}" name="Dia 10" dataDxfId="11"/>
+    <tableColumn id="13" xr3:uid="{E9D6ACAB-EF0B-42EB-977B-E157431B7C93}" name="Dia 11" dataDxfId="10"/>
+    <tableColumn id="14" xr3:uid="{7DE82C8F-4251-435F-8119-4098379E7C92}" name="Dia 12" dataDxfId="9"/>
+    <tableColumn id="15" xr3:uid="{C0057573-93FA-4291-8B0E-84DA468004AA}" name="Dia 13" dataDxfId="8"/>
+    <tableColumn id="16" xr3:uid="{616A7614-87CD-480E-8FB6-B3E991E2E773}" name="Dia 14" dataDxfId="7"/>
+    <tableColumn id="17" xr3:uid="{1EA39BE6-7D7D-43AD-8119-68FE10A2BB9C}" name="Dia 15" dataDxfId="6"/>
+    <tableColumn id="18" xr3:uid="{EF7A01F8-F878-4FFE-B140-126C702615BE}" name="Dia 16" dataDxfId="5"/>
+    <tableColumn id="19" xr3:uid="{9701BAD2-120F-49E8-9004-331E6F9C2716}" name="Dia 17" dataDxfId="4"/>
+    <tableColumn id="20" xr3:uid="{72A17F3E-6229-46C9-8FEE-BDF8B519F9FD}" name="Dia 18" dataDxfId="3"/>
+    <tableColumn id="21" xr3:uid="{1C3259A9-A4D5-488F-BE54-1D541CFA2C96}" name="Dia 19" dataDxfId="2"/>
+    <tableColumn id="22" xr3:uid="{4411E0A4-16AB-46BD-886B-34DA12503542}" name="Dia 20" dataDxfId="1"/>
+    <tableColumn id="23" xr3:uid="{4E8193E4-CA8B-435A-8A9E-B0AEB98006F5}" name="Horas pendentes" dataDxfId="0">
+      <calculatedColumnFormula>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2419,17 +2450,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V26"/>
+  <dimension ref="A1:W17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="91" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="11" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="12" max="21" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="19.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>23</v>
       </c>
@@ -2463,13 +2495,13 @@
       <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>12</v>
       </c>
       <c r="O1" s="1" t="s">
@@ -2496,8 +2528,11 @@
       <c r="V1" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="W1" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>24</v>
       </c>
@@ -2523,24 +2558,42 @@
         <v>2</v>
       </c>
       <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
+      <c r="L2" s="1">
+        <v>1</v>
+      </c>
       <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
+      <c r="N2" s="1">
+        <v>2</v>
+      </c>
       <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
+      <c r="P2" s="1">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>2</v>
+      </c>
+      <c r="R2" s="1">
+        <v>1</v>
+      </c>
       <c r="S2" s="1"/>
-      <c r="T2" s="1"/>
+      <c r="T2" s="1">
+        <v>2</v>
+      </c>
       <c r="U2" s="1"/>
-      <c r="V2" s="1"/>
+      <c r="V2" s="1">
+        <v>1</v>
+      </c>
+      <c r="W2" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B3" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
@@ -2556,20 +2609,28 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
+      <c r="K3" s="1">
+        <v>2</v>
+      </c>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
+      <c r="P3" s="1">
+        <v>2</v>
+      </c>
       <c r="Q3" s="1"/>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
+      <c r="W3" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
@@ -2602,8 +2663,12 @@
       <c r="T4" s="1"/>
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
+      <c r="W4" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>27</v>
       </c>
@@ -2632,8 +2697,12 @@
       <c r="T5" s="1"/>
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
+      <c r="W5" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
@@ -2664,8 +2733,12 @@
       <c r="T6" s="1"/>
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
+      <c r="W6" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>29</v>
       </c>
@@ -2694,8 +2767,12 @@
       <c r="T7" s="1"/>
       <c r="U7" s="1"/>
       <c r="V7" s="1"/>
+      <c r="W7" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>30</v>
       </c>
@@ -2716,8 +2793,12 @@
       </c>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
+      <c r="M8" s="1">
+        <v>2</v>
+      </c>
+      <c r="N8" s="1">
+        <v>0.5</v>
+      </c>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
@@ -2726,8 +2807,12 @@
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
+      <c r="W8" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>31</v>
       </c>
@@ -2756,8 +2841,12 @@
       <c r="T9" s="1"/>
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
+      <c r="W9" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>32</v>
       </c>
@@ -2778,9 +2867,13 @@
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
+      <c r="M10" s="1">
+        <v>3</v>
+      </c>
       <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
+      <c r="O10" s="1">
+        <v>2.5</v>
+      </c>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
@@ -2788,13 +2881,17 @@
       <c r="T10" s="1"/>
       <c r="U10" s="1"/>
       <c r="V10" s="1"/>
+      <c r="W10" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -2818,13 +2915,17 @@
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
+      <c r="W11" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B12" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -2834,22 +2935,34 @@
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1">
-        <v>1.5</v>
-      </c>
-      <c r="K12" s="1"/>
+        <v>3</v>
+      </c>
+      <c r="K12" s="1">
+        <v>2</v>
+      </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="1"/>
-      <c r="Q12" s="1"/>
+      <c r="O12" s="1">
+        <v>2</v>
+      </c>
+      <c r="P12" s="1">
+        <v>2</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>1</v>
+      </c>
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
+      <c r="W12" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>35</v>
       </c>
@@ -2869,7 +2982,9 @@
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
+      <c r="N13" s="1">
+        <v>1</v>
+      </c>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
       <c r="Q13" s="1"/>
@@ -2878,8 +2993,12 @@
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
+      <c r="W13" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>36</v>
       </c>
@@ -2894,25 +3013,33 @@
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
+      <c r="K14" s="1">
+        <v>3</v>
+      </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
+      <c r="P14" s="1">
+        <v>2</v>
+      </c>
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
+      <c r="W14" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B15" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -2929,407 +3056,199 @@
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
+      <c r="P15" s="1">
+        <v>1.5</v>
+      </c>
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
+      <c r="W15" s="1">
+        <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
-      <c r="Q16" s="1"/>
-      <c r="R16" s="1"/>
-      <c r="S16" s="1"/>
-      <c r="T16" s="1"/>
-      <c r="U16" s="1"/>
-      <c r="V16" s="1"/>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="9">
+        <f>SUM(B2:B15)</f>
+        <v>74</v>
+      </c>
+      <c r="C16" s="6">
+        <f>B16-SUM(C2:C15)</f>
+        <v>64</v>
+      </c>
+      <c r="D16" s="6">
+        <f>C16-SUM(D2:D15)</f>
+        <v>61</v>
+      </c>
+      <c r="E16" s="6">
+        <f>D16-SUM(E2:E15)</f>
+        <v>58</v>
+      </c>
+      <c r="F16" s="6">
+        <f>E16-SUM(F2:F15)</f>
+        <v>51</v>
+      </c>
+      <c r="G16" s="6">
+        <f>F16-SUM(G2:G15)</f>
+        <v>50</v>
+      </c>
+      <c r="H16" s="6">
+        <f>G16-SUM(H2:H15)</f>
+        <v>50</v>
+      </c>
+      <c r="I16" s="9">
+        <f>H16-SUM(I2:I15)</f>
+        <v>49</v>
+      </c>
+      <c r="J16" s="6">
+        <f>I16-SUM(J2:J15)</f>
+        <v>37.5</v>
+      </c>
+      <c r="K16" s="6">
+        <f>J16-SUM(K2:K15)</f>
+        <v>30.5</v>
+      </c>
+      <c r="L16" s="9">
+        <f>K16-SUM(L2:L15)</f>
+        <v>29.5</v>
+      </c>
+      <c r="M16" s="6">
+        <f>L16-SUM(M2:M15)</f>
+        <v>24.5</v>
+      </c>
+      <c r="N16" s="6">
+        <f>M16-SUM(N2:N15)</f>
+        <v>21</v>
+      </c>
+      <c r="O16" s="6">
+        <f>N16-SUM(O2:O15)</f>
+        <v>16.5</v>
+      </c>
+      <c r="P16" s="6">
+        <f>O16-SUM(P2:P15)</f>
+        <v>7</v>
+      </c>
+      <c r="Q16" s="6">
+        <f>P16-SUM(Q2:Q15)</f>
+        <v>4</v>
+      </c>
+      <c r="R16" s="6">
+        <f>Q16-SUM(R2:R15)</f>
+        <v>3</v>
+      </c>
+      <c r="S16" s="6">
+        <f>R16-SUM(S2:S15)</f>
+        <v>3</v>
+      </c>
+      <c r="T16" s="6">
+        <f>S16-SUM(T2:T15)</f>
+        <v>1</v>
+      </c>
+      <c r="U16" s="6">
+        <f>T16-SUM(U2:U15)</f>
+        <v>1</v>
+      </c>
+      <c r="V16" s="6">
+        <f>U16-SUM(V2:V15)</f>
+        <v>0</v>
+      </c>
+      <c r="W16" s="1"/>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A17" s="2"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
-      <c r="Q17" s="1"/>
-      <c r="R17" s="1"/>
-      <c r="S17" s="1"/>
-      <c r="T17" s="1"/>
-      <c r="U17" s="1"/>
-      <c r="V17" s="1"/>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A18" s="2"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
-      <c r="Q18" s="1"/>
-      <c r="R18" s="1"/>
-      <c r="S18" s="1"/>
-      <c r="T18" s="1"/>
-      <c r="U18" s="1"/>
-      <c r="V18" s="1"/>
-    </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A19" s="2"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
-      <c r="Q19" s="1"/>
-      <c r="R19" s="1"/>
-      <c r="S19" s="1"/>
-      <c r="T19" s="1"/>
-      <c r="U19" s="1"/>
-      <c r="V19" s="1"/>
-    </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A20" s="2"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
-      <c r="P20" s="1"/>
-      <c r="Q20" s="1"/>
-      <c r="R20" s="1"/>
-      <c r="S20" s="1"/>
-      <c r="T20" s="1"/>
-      <c r="U20" s="1"/>
-      <c r="V20" s="1"/>
-    </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A21" s="2"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-      <c r="P21" s="1"/>
-      <c r="Q21" s="1"/>
-      <c r="R21" s="1"/>
-      <c r="S21" s="1"/>
-      <c r="T21" s="1"/>
-      <c r="U21" s="1"/>
-      <c r="V21" s="1"/>
-    </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A22" s="2"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
-      <c r="P22" s="1"/>
-      <c r="Q22" s="1"/>
-      <c r="R22" s="1"/>
-      <c r="S22" s="1"/>
-      <c r="T22" s="1"/>
-      <c r="U22" s="1"/>
-      <c r="V22" s="1"/>
-    </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A23" s="2"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
-      <c r="P23" s="1"/>
-      <c r="Q23" s="1"/>
-      <c r="R23" s="1"/>
-      <c r="S23" s="1"/>
-      <c r="T23" s="1"/>
-      <c r="U23" s="1"/>
-      <c r="V23" s="1"/>
-    </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A24" s="2"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-      <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
-      <c r="N24" s="1"/>
-      <c r="O24" s="1"/>
-      <c r="P24" s="1"/>
-      <c r="Q24" s="1"/>
-      <c r="R24" s="1"/>
-      <c r="S24" s="2"/>
-      <c r="T24" s="1"/>
-      <c r="U24" s="1"/>
-      <c r="V24" s="1"/>
-    </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" s="4">
-        <f>SUM(B2:B24)</f>
-        <v>83</v>
-      </c>
-      <c r="C25" s="4">
-        <f t="shared" ref="C25:V25" si="0">B25-SUM(C2:C24)</f>
-        <v>73</v>
-      </c>
-      <c r="D25" s="4">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="8">
+        <f>SUM(B2:B15)</f>
+        <v>74</v>
+      </c>
+      <c r="C17" s="7">
+        <f>$B$17-(($B$17/20)*(COLUMN()-2))</f>
+        <v>70.3</v>
+      </c>
+      <c r="D17" s="7">
+        <f t="shared" ref="D17:V17" si="0">$B$17-(($B$17/20)*(COLUMN()-2))</f>
+        <v>66.599999999999994</v>
+      </c>
+      <c r="E17" s="7">
         <f t="shared" si="0"/>
-        <v>70</v>
-      </c>
-      <c r="E25" s="4">
+        <v>62.9</v>
+      </c>
+      <c r="F17" s="7">
         <f t="shared" si="0"/>
-        <v>67</v>
-      </c>
-      <c r="F25" s="4">
+        <v>59.2</v>
+      </c>
+      <c r="G17" s="7">
         <f t="shared" si="0"/>
-        <v>60</v>
-      </c>
-      <c r="G25" s="4">
+        <v>55.5</v>
+      </c>
+      <c r="H17" s="7">
         <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-      <c r="H25" s="4">
+        <v>51.8</v>
+      </c>
+      <c r="I17" s="7">
         <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-      <c r="I25" s="4">
-        <f>H25-SUM(I2:I24)</f>
-        <v>58</v>
-      </c>
-      <c r="J25" s="4">
+        <v>48.099999999999994</v>
+      </c>
+      <c r="J17" s="7">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="K25" s="4">
+        <v>44.4</v>
+      </c>
+      <c r="K17" s="7">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="L25" s="4">
-        <f>K25-SUM(L2:L24)</f>
-        <v>48</v>
-      </c>
-      <c r="M25" s="4">
+        <v>40.699999999999996</v>
+      </c>
+      <c r="L17" s="7">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="N25" s="4">
+        <v>37</v>
+      </c>
+      <c r="M17" s="7">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="O25" s="4">
+        <v>33.299999999999997</v>
+      </c>
+      <c r="N17" s="7">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="P25" s="4">
+        <v>29.599999999999994</v>
+      </c>
+      <c r="O17" s="7">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="Q25" s="4">
+        <v>25.9</v>
+      </c>
+      <c r="P17" s="7">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="R25" s="4">
+        <v>22.199999999999996</v>
+      </c>
+      <c r="Q17" s="7">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="S25" s="4">
+        <v>18.5</v>
+      </c>
+      <c r="R17" s="7">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="T25" s="4">
+        <v>14.799999999999997</v>
+      </c>
+      <c r="S17" s="7">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="U25" s="4">
+        <v>11.099999999999994</v>
+      </c>
+      <c r="T17" s="7">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="V25" s="4">
+        <v>7.3999999999999915</v>
+      </c>
+      <c r="U17" s="7">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B26" s="6">
-        <f>SUM(B2:B24)</f>
-        <v>83</v>
-      </c>
-      <c r="C26" s="6">
-        <f>$B$26-(($B$26/20)*(COLUMN()-2))</f>
-        <v>78.849999999999994</v>
-      </c>
-      <c r="D26" s="6">
-        <f t="shared" ref="D26:V26" si="1">$B$26-(($B$26/20)*(COLUMN()-2))</f>
-        <v>74.7</v>
-      </c>
-      <c r="E26" s="6">
-        <f t="shared" si="1"/>
-        <v>70.55</v>
-      </c>
-      <c r="F26" s="6">
-        <f t="shared" si="1"/>
-        <v>66.400000000000006</v>
-      </c>
-      <c r="G26" s="6">
-        <f t="shared" si="1"/>
-        <v>62.25</v>
-      </c>
-      <c r="H26" s="6">
-        <f t="shared" si="1"/>
-        <v>58.099999999999994</v>
-      </c>
-      <c r="I26" s="6">
-        <f t="shared" si="1"/>
-        <v>53.949999999999996</v>
-      </c>
-      <c r="J26" s="6">
-        <f t="shared" si="1"/>
-        <v>49.8</v>
-      </c>
-      <c r="K26" s="6">
-        <f t="shared" si="1"/>
-        <v>45.65</v>
-      </c>
-      <c r="L26" s="6">
-        <f t="shared" si="1"/>
-        <v>41.5</v>
-      </c>
-      <c r="M26" s="6">
-        <f t="shared" si="1"/>
-        <v>37.349999999999994</v>
-      </c>
-      <c r="N26" s="6">
-        <f t="shared" si="1"/>
-        <v>33.199999999999996</v>
-      </c>
-      <c r="O26" s="6">
-        <f t="shared" si="1"/>
-        <v>29.049999999999997</v>
-      </c>
-      <c r="P26" s="6">
-        <f t="shared" si="1"/>
-        <v>24.899999999999991</v>
-      </c>
-      <c r="Q26" s="6">
-        <f t="shared" si="1"/>
-        <v>20.749999999999993</v>
-      </c>
-      <c r="R26" s="6">
-        <f t="shared" si="1"/>
-        <v>16.599999999999994</v>
-      </c>
-      <c r="S26" s="6">
-        <f t="shared" si="1"/>
-        <v>12.449999999999989</v>
-      </c>
-      <c r="T26" s="6">
-        <f t="shared" si="1"/>
-        <v>8.2999999999999972</v>
-      </c>
-      <c r="U26" s="6">
-        <f t="shared" si="1"/>
-        <v>4.1499999999999915</v>
-      </c>
-      <c r="V26" s="6">
-        <f t="shared" si="1"/>
+        <v>3.7000000000000028</v>
+      </c>
+      <c r="V17" s="7">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="W17" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>